<commit_message>
submit task report week 3
</commit_message>
<xml_diff>
--- a/GroupTaskReport.xlsx
+++ b/GroupTaskReport.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\project-rbl-swd392_group2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\project-rbl-1-swd392_se19b06_group2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CBBFB3-7BA4-4713-958E-CC5F3441CA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C615A984-670A-4821-B455-440A19F5818E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
+    <sheet name="Week 3" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>Member</t>
   </si>
@@ -63,6 +64,21 @@
   <si>
     <t>Update use case diagram với secondary actor (AI Prediction Service &amp; Payment Gateway)
 Cập nhật use case diagrams và chuẩn hóa mối quan hệ giữa các diagrams.</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram AI Prediction &amp; Recommendation</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Authentication &amp; User Management</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Order Management &amp; Payment Management</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Dashboard &amp; Analytics</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Menu Management</t>
   </si>
 </sst>
 </file>
@@ -473,4 +489,66 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{218B877B-1C84-4135-817C-4F22A1135DD4}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.8125" customWidth="1"/>
+    <col min="2" max="2" width="62.4375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="14.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
submit report week 4
</commit_message>
<xml_diff>
--- a/GroupTaskReport.xlsx
+++ b/GroupTaskReport.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\project-rbl-1-swd392_se19b06_group2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C615A984-670A-4821-B455-440A19F5818E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCD8391-CBC3-4584-8FAB-784CBAA9B9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="2" r:id="rId2"/>
+    <sheet name="Week 4" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t>Member</t>
   </si>
@@ -79,6 +80,21 @@
   </si>
   <si>
     <t>Vẽ Class Diagram Menu Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams Schedule Menu Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams Daily Menu Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams Authentication &amp; User Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams Food Item &amp; Category Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams Order Management</t>
   </si>
 </sst>
 </file>
@@ -551,4 +567,66 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF860916-3951-46EA-9713-2800C9C3F4F7}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.375" customWidth="1"/>
+    <col min="2" max="2" width="44.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="14.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
submit report week 5
</commit_message>
<xml_diff>
--- a/GroupTaskReport.xlsx
+++ b/GroupTaskReport.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\project-rbl-1-swd392_se19b06_group2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCD8391-CBC3-4584-8FAB-784CBAA9B9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D2861D-830B-408C-BE0F-6A8E5432B775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="2" r:id="rId2"/>
     <sheet name="Week 4" sheetId="3" r:id="rId3"/>
+    <sheet name="Week 5" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
   <si>
     <t>Member</t>
   </si>
@@ -95,6 +96,21 @@
   </si>
   <si>
     <t>Vẽ Sequence Diagrams Order Management</t>
+  </si>
+  <si>
+    <t>Tiếp tục vẽ Sequence Diagrams Schedule Menu Management</t>
+  </si>
+  <si>
+    <t>Tiếp tục vẽ Sequence Diagrams Daily Menu Management</t>
+  </si>
+  <si>
+    <t>Tiếp tục vẽ Sequence Diagrams Authentication &amp; User Management</t>
+  </si>
+  <si>
+    <t>Tiếp tục vẽ Sequence Diagrams Food Item &amp; Category Management</t>
+  </si>
+  <si>
+    <t>Tiếp tục vẽ Sequence Diagrams Order Management</t>
   </si>
 </sst>
 </file>
@@ -629,4 +645,66 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD869BD-EF8A-4630-AEDA-3C0B2E22936B}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.6875" customWidth="1"/>
+    <col min="2" max="2" width="61.3125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="14.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
submit report week 7
</commit_message>
<xml_diff>
--- a/GroupTaskReport.xlsx
+++ b/GroupTaskReport.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yna\Study\TERM_7\SWD392\project-rbl-1-swd392_se19b06_group2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D2861D-830B-408C-BE0F-6A8E5432B775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F1C153E-69DE-40AF-AF17-BE6A9990876E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="2" r:id="rId2"/>
     <sheet name="Week 4" sheetId="3" r:id="rId3"/>
     <sheet name="Week 5" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 6" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
   <si>
     <t>Member</t>
   </si>
@@ -68,49 +69,49 @@
 Cập nhật use case diagrams và chuẩn hóa mối quan hệ giữa các diagrams.</t>
   </si>
   <si>
-    <t>Vẽ Class Diagram AI Prediction &amp; Recommendation</t>
-  </si>
-  <si>
-    <t>Vẽ Class Diagram Authentication &amp; User Management</t>
-  </si>
-  <si>
-    <t>Vẽ Class Diagram Order Management &amp; Payment Management</t>
-  </si>
-  <si>
-    <t>Vẽ Class Diagram Dashboard &amp; Analytics</t>
-  </si>
-  <si>
-    <t>Vẽ Class Diagram Menu Management</t>
-  </si>
-  <si>
-    <t>Vẽ Sequence Diagrams Schedule Menu Management</t>
-  </si>
-  <si>
-    <t>Vẽ Sequence Diagrams Daily Menu Management</t>
-  </si>
-  <si>
-    <t>Vẽ Sequence Diagrams Authentication &amp; User Management</t>
-  </si>
-  <si>
-    <t>Vẽ Sequence Diagrams Food Item &amp; Category Management</t>
-  </si>
-  <si>
-    <t>Vẽ Sequence Diagrams Order Management</t>
-  </si>
-  <si>
-    <t>Tiếp tục vẽ Sequence Diagrams Schedule Menu Management</t>
-  </si>
-  <si>
-    <t>Tiếp tục vẽ Sequence Diagrams Daily Menu Management</t>
-  </si>
-  <si>
-    <t>Tiếp tục vẽ Sequence Diagrams Authentication &amp; User Management</t>
-  </si>
-  <si>
-    <t>Tiếp tục vẽ Sequence Diagrams Food Item &amp; Category Management</t>
-  </si>
-  <si>
-    <t>Tiếp tục vẽ Sequence Diagrams Order Management</t>
+    <t>Vẽ Class Diagram Daily Menu Management &amp; AI Prediction &amp; Recommendation</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Schedule Menu Management &amp; Notification Management</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Authentication, User Management &amp; Payment Management</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Category &amp; Food Item Management, Analytics &amp; Reporting</t>
+  </si>
+  <si>
+    <t>Vẽ Class Diagram Order Management</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams cho UC Login, Logout, Create User Account, View Personal Profile, Process Payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vẽ Sequence Diagrams cho UC Create Order, Cancel Order, View Order List, </t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams cho UC Create Food Item, Configure Food Category, View Daily Revenue</t>
+  </si>
+  <si>
+    <t>Vẽ Sequence Diagrams cho UC Configure Scheduled Menu, View Scheduled Menu, View Notifications, Mark Notification as Read</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vẽ Sequence Diagrams cho UC Update Daily Menu Item, View Food Demand Forecast, View Dynamic Pricing Recommendation, Apply Recommended Daily Quantity, </t>
+  </si>
+  <si>
+    <t>Vẽ Communication Diagrams cho UC Configure Scheduled Menu, View Scheduled Menu, View Notifications, Mark Notification as Read</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vẽ Communication Diagrams cho UC Update Daily Menu Item, View Food Demand Forecast, View Dynamic Pricing Recommendation, Apply Recommended Daily Quantity, </t>
+  </si>
+  <si>
+    <t>Vẽ Communication Diagrams cho UC Login, Logout, Create User Account, View Personal Profile, Process Payment</t>
+  </si>
+  <si>
+    <t>Vẽ Communication Diagrams cho UC Create Food Item, Configure Food Category, View Daily Revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vẽ Communication Diagrams cho UC Create Order, Cancel Order, View Order List, </t>
   </si>
 </sst>
 </file>
@@ -540,23 +541,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -564,7 +565,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -590,8 +591,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.375" customWidth="1"/>
-    <col min="2" max="2" width="44.875" customWidth="1"/>
+    <col min="1" max="1" width="28.3125" customWidth="1"/>
+    <col min="2" max="2" width="63.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="14.25" thickBot="1" x14ac:dyDescent="0.4">
@@ -602,20 +603,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" ht="40.9" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="40.9" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
@@ -623,7 +624,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
@@ -631,15 +632,15 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -664,7 +665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -672,7 +673,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" ht="40.9" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -680,7 +681,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -688,7 +689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -696,7 +697,69 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="13.9" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0290115-AC4A-45F7-A60B-5191D62DB410}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.6875" customWidth="1"/>
+    <col min="2" max="2" width="61.3125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="14.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="40.9" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="27.4" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>

</xml_diff>